<commit_message>
Re-run every complete-network analysis on the deduplicated graph (v1.6.0)
The complete TRON USDT network was rebuilt with duplicate event rows removed
(2,375,557,775 rows, 2,225,933,042 distinct transfers) and every analysis that
reads it was re-run. Address set, pair set and all connectivity results are
byte-identical; value sums fall by about seven per cent (total 14.43 trillion
USDT; value incident to the designated addresses 9.94 billion, now equal to the
per-address histories; stranded value for the 400/1,000/10,000 highest-degree
undesignated addresses 3.15/4.70/8.98 billion). Adds the exact distinct-transfer
count, the streaming graph builder, the old-versus-new comparison script and a
two-phase mode for the degree-matched interval.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Source_Data.xlsx
+++ b/Source_Data.xlsx
@@ -830,7 +830,7 @@
         <v>0.002263103458721716</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06871602063158783</v>
+        <v>0.06884952128720195</v>
       </c>
       <c r="D2" t="n">
         <v>590</v>
@@ -852,10 +852,10 @@
         <v>0.002117764705670593</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01776209622083104</v>
+        <v>0.01793006064507883</v>
       </c>
       <c r="D3" t="n">
-        <v>7653.089873999999</v>
+        <v>12191.25990994771</v>
       </c>
       <c r="E3" t="n">
         <v>0.001269778531743261</v>
@@ -864,16 +864,16 @@
         <v>0.003962613216382103</v>
       </c>
       <c r="G3" t="n">
-        <v>0.009863726585278258</v>
+        <v>0.0100252989463729</v>
       </c>
       <c r="H3" t="n">
-        <v>0.03174847599774792</v>
+        <v>0.03193038036053411</v>
       </c>
       <c r="I3" t="n">
-        <v>3167.649748</v>
+        <v>3094.649741172791</v>
       </c>
       <c r="J3" t="n">
-        <v>12138.53</v>
+        <v>21340.59976935387</v>
       </c>
     </row>
     <row r="4">
@@ -904,10 +904,10 @@
         <v>26.87325854076248</v>
       </c>
       <c r="C5" t="n">
-        <v>44.94682669335663</v>
+        <v>44.35256530000485</v>
       </c>
       <c r="D5" t="n">
-        <v>3414178773.126534</v>
+        <v>3154012306.778911</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -926,10 +926,10 @@
         <v>34.23216946127282</v>
       </c>
       <c r="C6" t="n">
-        <v>47.06389967847252</v>
+        <v>46.48448414237567</v>
       </c>
       <c r="D6" t="n">
-        <v>5044081470.875386</v>
+        <v>4696813960.444774</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -948,10 +948,10 @@
         <v>48.3707159399376</v>
       </c>
       <c r="C7" t="n">
-        <v>54.28443105166888</v>
+        <v>53.81360211389838</v>
       </c>
       <c r="D7" t="n">
-        <v>9605729803.472935</v>
+        <v>8975320466.222982</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>

</xml_diff>